<commit_message>
1st model of the day
</commit_message>
<xml_diff>
--- a/compareOP.xlsx
+++ b/compareOP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DUT\Ki 2\Edge AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43AB01B8-2417-449C-BF5D-DFEE8E2BC276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E64CC8D-0935-4854-B2C3-17FA4CC13C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56603411-7B59-498E-88B9-7E9448248F05}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>Pct</t>
   </si>
   <si>
-    <t>Gemini.1</t>
-  </si>
-  <si>
     <t>V</t>
   </si>
   <si>
@@ -49,10 +46,14 @@
   </si>
   <si>
     <t>Gem1
-25% val</t>
+Custom</t>
   </si>
   <si>
-    <t>Gem1
+    <t>Gem2
+Custom</t>
+  </si>
+  <si>
+    <t>Gemini.1
 Custom</t>
   </si>
 </sst>
@@ -139,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -158,10 +159,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1023,8 +1027,8 @@
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>8</v>
+      <c r="C1" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
@@ -1032,7 +1036,7 @@
       <c r="G1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1044,7 +1048,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="6"/>
       <c r="F2">
@@ -1062,7 +1066,7 @@
       </c>
       <c r="L2" s="4">
         <f>COUNTIF(I2:I1001, "T")</f>
-        <v>1000</v>
+        <v>936</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1073,7 +1077,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="6"/>
       <c r="F3">
@@ -1091,7 +1095,7 @@
       </c>
       <c r="L3" s="4">
         <f>L2/1000*100</f>
-        <v>100</v>
+        <v>93.600000000000009</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
@@ -1102,7 +1106,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="6"/>
       <c r="F4">
@@ -1124,18 +1128,18 @@
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="6"/>
       <c r="F5">
         <v>14</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I5" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
@@ -1146,7 +1150,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="6"/>
       <c r="F6">
@@ -1168,7 +1172,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6"/>
       <c r="F7">
@@ -1190,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="6"/>
       <c r="F8">
@@ -1212,7 +1216,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="6"/>
       <c r="F9">
@@ -1249,7 +1253,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D10" s="6"/>
       <c r="F10">
@@ -1271,7 +1275,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11" s="6"/>
       <c r="F11">
@@ -1293,7 +1297,7 @@
         <v>7</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="6"/>
       <c r="F12">
@@ -1315,7 +1319,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D13" s="6"/>
       <c r="F13">
@@ -1337,7 +1341,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="6"/>
       <c r="F14">
@@ -1359,7 +1363,7 @@
         <v>7</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" s="6"/>
       <c r="F15">
@@ -1381,7 +1385,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D16" s="6"/>
       <c r="F16">
@@ -1418,7 +1422,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D17" s="6"/>
       <c r="F17">
@@ -1441,7 +1445,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D18" s="6"/>
       <c r="F18">
@@ -1463,24 +1467,24 @@
         <v>1</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" s="6"/>
       <c r="F19">
         <v>59</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I19" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
-      </c>
-      <c r="O19" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
+        <v>F</v>
+      </c>
+      <c r="O19" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="P19" s="9"/>
+      <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
@@ -1492,16 +1496,18 @@
       <c r="C20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="6"/>
+      <c r="D20" s="6">
+        <v>6</v>
+      </c>
       <c r="F20">
         <v>63</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
@@ -1512,7 +1518,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D21" s="6">
         <v>1</v>
@@ -1521,11 +1527,11 @@
         <v>67</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
@@ -1536,7 +1542,7 @@
         <v>5</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="6"/>
       <c r="F22">
@@ -1558,18 +1564,18 @@
         <v>6</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="6"/>
       <c r="F23">
         <v>70</v>
       </c>
       <c r="G23">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I23" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
@@ -1580,7 +1586,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="6"/>
       <c r="F24">
@@ -1602,7 +1608,7 @@
         <v>6</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="6"/>
       <c r="F25">
@@ -1624,7 +1630,7 @@
         <v>9</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" s="6"/>
       <c r="F26">
@@ -1646,7 +1652,7 @@
         <v>6</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" s="6"/>
       <c r="F27">
@@ -1668,7 +1674,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D28" s="6"/>
       <c r="F28">
@@ -1690,7 +1696,7 @@
         <v>6</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="6"/>
       <c r="F29">
@@ -1712,7 +1718,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D30" s="6"/>
       <c r="F30">
@@ -1734,7 +1740,7 @@
         <v>3</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="6"/>
       <c r="F31">
@@ -1756,7 +1762,7 @@
         <v>2</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D32" s="6"/>
       <c r="F32">
@@ -1778,7 +1784,7 @@
         <v>5</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="6"/>
       <c r="F33">
@@ -1800,7 +1806,7 @@
         <v>5</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D34" s="6"/>
       <c r="F34">
@@ -1822,7 +1828,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="6"/>
       <c r="F35">
@@ -1844,7 +1850,7 @@
         <v>3</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="6"/>
       <c r="F36">
@@ -1866,7 +1872,7 @@
         <v>2</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D37" s="6"/>
       <c r="F37">
@@ -1888,7 +1894,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D38" s="6"/>
       <c r="F38">
@@ -1910,7 +1916,7 @@
         <v>3</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D39" s="6"/>
       <c r="F39">
@@ -1932,7 +1938,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D40" s="6"/>
       <c r="F40">
@@ -1954,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D41" s="6"/>
       <c r="F41">
@@ -1976,7 +1982,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D42" s="6"/>
       <c r="F42">
@@ -1998,7 +2004,7 @@
         <v>4</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D43" s="6"/>
       <c r="F43">
@@ -2020,7 +2026,7 @@
         <v>6</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D44" s="6"/>
       <c r="F44">
@@ -2042,7 +2048,7 @@
         <v>3</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D45" s="6"/>
       <c r="F45">
@@ -2064,7 +2070,7 @@
         <v>6</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D46" s="6"/>
       <c r="F46">
@@ -2086,7 +2092,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D47" s="6"/>
       <c r="F47">
@@ -2108,7 +2114,7 @@
         <v>2</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48" s="6"/>
       <c r="F48">
@@ -2130,7 +2136,7 @@
         <v>3</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D49" s="6"/>
       <c r="F49">
@@ -2152,7 +2158,7 @@
         <v>7</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D50" s="6"/>
       <c r="F50">
@@ -2174,7 +2180,7 @@
         <v>2</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D51" s="6"/>
       <c r="F51">
@@ -2196,7 +2202,7 @@
         <v>6</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D52" s="6"/>
       <c r="F52">
@@ -2218,7 +2224,7 @@
         <v>6</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D53" s="6"/>
       <c r="F53">
@@ -2240,7 +2246,7 @@
         <v>3</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D54" s="6"/>
       <c r="F54">
@@ -2262,7 +2268,7 @@
         <v>5</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D55" s="6"/>
       <c r="F55">
@@ -2284,7 +2290,7 @@
         <v>2</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D56" s="6"/>
       <c r="F56">
@@ -2306,7 +2312,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D57" s="6"/>
       <c r="F57">
@@ -2328,7 +2334,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D58" s="6"/>
       <c r="F58">
@@ -2350,7 +2356,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D59" s="6"/>
       <c r="F59">
@@ -2372,7 +2378,7 @@
         <v>2</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D60" s="6"/>
       <c r="F60">
@@ -2394,7 +2400,7 @@
         <v>2</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D61" s="6"/>
       <c r="F61">
@@ -2416,7 +2422,7 @@
         <v>6</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" s="6"/>
       <c r="F62">
@@ -2438,7 +2444,7 @@
         <v>2</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D63" s="6"/>
       <c r="F63">
@@ -2460,7 +2466,7 @@
         <v>2</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D64" s="6"/>
       <c r="F64">
@@ -2482,7 +2488,7 @@
         <v>4</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D65" s="6"/>
       <c r="F65">
@@ -2504,7 +2510,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D66" s="6"/>
       <c r="F66">
@@ -2526,7 +2532,7 @@
         <v>0</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D67" s="6"/>
       <c r="F67">
@@ -2548,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D68" s="6"/>
       <c r="F68">
@@ -2570,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D69" s="6"/>
       <c r="F69">
@@ -2592,7 +2598,7 @@
         <v>6</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D70" s="6"/>
       <c r="F70">
@@ -2614,7 +2620,7 @@
         <v>6</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D71" s="6"/>
       <c r="F71">
@@ -2636,7 +2642,7 @@
         <v>4</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D72" s="6"/>
       <c r="F72">
@@ -2658,7 +2664,7 @@
         <v>4</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D73" s="6"/>
       <c r="F73">
@@ -2680,7 +2686,7 @@
         <v>0</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D74" s="6"/>
       <c r="F74">
@@ -2702,7 +2708,7 @@
         <v>2</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D75" s="6"/>
       <c r="F75">
@@ -2724,7 +2730,7 @@
         <v>2</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D76" s="6"/>
       <c r="F76">
@@ -2746,7 +2752,7 @@
         <v>1</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D77" s="6"/>
       <c r="F77">
@@ -2768,7 +2774,7 @@
         <v>0</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D78" s="6"/>
       <c r="F78">
@@ -2790,7 +2796,7 @@
         <v>2</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D79" s="6">
         <v>6</v>
@@ -2799,11 +2805,11 @@
         <v>229</v>
       </c>
       <c r="G79">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I79" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
@@ -2814,7 +2820,7 @@
         <v>5</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D80" s="6"/>
       <c r="F80">
@@ -2836,7 +2842,7 @@
         <v>2</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D81" s="6"/>
       <c r="F81">
@@ -2858,7 +2864,7 @@
         <v>2</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D82" s="6"/>
       <c r="F82">
@@ -2880,7 +2886,7 @@
         <v>1</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D83" s="6"/>
       <c r="F83">
@@ -2902,7 +2908,7 @@
         <v>2</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D84" s="6"/>
       <c r="F84">
@@ -2924,7 +2930,7 @@
         <v>2</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D85" s="6"/>
       <c r="F85">
@@ -2946,7 +2952,7 @@
         <v>1</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D86" s="6"/>
       <c r="F86">
@@ -2968,7 +2974,7 @@
         <v>1</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D87" s="6"/>
       <c r="F87">
@@ -2990,7 +2996,7 @@
         <v>6</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D88" s="6"/>
       <c r="F88">
@@ -3012,7 +3018,7 @@
         <v>6</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D89" s="6"/>
       <c r="F89">
@@ -3034,7 +3040,7 @@
         <v>0</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D90" s="6"/>
       <c r="F90">
@@ -3056,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D91" s="6"/>
       <c r="F91">
@@ -3078,7 +3084,7 @@
         <v>2</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D92" s="6"/>
       <c r="F92">
@@ -3100,7 +3106,7 @@
         <v>1</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D93" s="6"/>
       <c r="F93">
@@ -3122,7 +3128,7 @@
         <v>0</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D94" s="6"/>
       <c r="F94">
@@ -3144,7 +3150,7 @@
         <v>5</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D95" s="6"/>
       <c r="F95">
@@ -3166,7 +3172,7 @@
         <v>0</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D96" s="6"/>
       <c r="F96">
@@ -3188,7 +3194,7 @@
         <v>2</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D97" s="6"/>
       <c r="F97">
@@ -3210,7 +3216,7 @@
         <v>1</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D98" s="6"/>
       <c r="F98">
@@ -3232,7 +3238,7 @@
         <v>0</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D99" s="6"/>
       <c r="F99">
@@ -3254,7 +3260,7 @@
         <v>6</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D100" s="6"/>
       <c r="F100">
@@ -3276,7 +3282,7 @@
         <v>6</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D101" s="6"/>
       <c r="F101">
@@ -3298,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D102" s="6"/>
       <c r="F102">
@@ -3320,18 +3326,18 @@
         <v>6</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D103" s="6"/>
       <c r="F103">
         <v>282</v>
       </c>
       <c r="G103">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I103" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.3">
@@ -3342,7 +3348,7 @@
         <v>9</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D104" s="6"/>
       <c r="F104">
@@ -3364,7 +3370,7 @@
         <v>9</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D105" s="6"/>
       <c r="F105">
@@ -3386,7 +3392,7 @@
         <v>1</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D106" s="6"/>
       <c r="F106">
@@ -3408,7 +3414,7 @@
         <v>4</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D107" s="6"/>
       <c r="F107">
@@ -3430,7 +3436,7 @@
         <v>2</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D108" s="6"/>
       <c r="F108">
@@ -3452,7 +3458,7 @@
         <v>5</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D109" s="6"/>
       <c r="F109">
@@ -3474,7 +3480,7 @@
         <v>8</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D110" s="6"/>
       <c r="F110">
@@ -3496,7 +3502,7 @@
         <v>1</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D111" s="6"/>
       <c r="F111">
@@ -3518,7 +3524,7 @@
         <v>3</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D112" s="6"/>
       <c r="F112">
@@ -3540,7 +3546,7 @@
         <v>2</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D113" s="6"/>
       <c r="F113">
@@ -3562,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D114" s="6"/>
       <c r="F114">
@@ -3584,7 +3590,7 @@
         <v>1</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D115" s="6"/>
       <c r="F115">
@@ -3606,7 +3612,7 @@
         <v>1</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D116" s="6"/>
       <c r="F116">
@@ -3628,7 +3634,7 @@
         <v>1</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D117" s="6"/>
       <c r="F117">
@@ -3650,7 +3656,7 @@
         <v>1</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D118" s="6"/>
       <c r="F118">
@@ -3672,7 +3678,7 @@
         <v>0</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D119" s="6"/>
       <c r="F119">
@@ -3694,7 +3700,7 @@
         <v>0</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D120" s="6"/>
       <c r="F120">
@@ -3716,7 +3722,7 @@
         <v>2</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D121" s="6"/>
       <c r="F121">
@@ -3738,7 +3744,7 @@
         <v>6</v>
       </c>
       <c r="C122" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D122" s="6"/>
       <c r="F122">
@@ -3760,7 +3766,7 @@
         <v>3</v>
       </c>
       <c r="C123" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D123" s="6"/>
       <c r="F123">
@@ -3782,7 +3788,7 @@
         <v>2</v>
       </c>
       <c r="C124" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D124" s="6"/>
       <c r="F124">
@@ -3804,7 +3810,7 @@
         <v>2</v>
       </c>
       <c r="C125" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D125" s="6"/>
       <c r="F125">
@@ -3826,7 +3832,7 @@
         <v>1</v>
       </c>
       <c r="C126" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D126" s="6"/>
       <c r="F126">
@@ -3848,7 +3854,7 @@
         <v>1</v>
       </c>
       <c r="C127" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D127" s="6"/>
       <c r="F127">
@@ -3870,7 +3876,7 @@
         <v>0</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D128" s="6"/>
       <c r="F128">
@@ -3892,7 +3898,7 @@
         <v>1</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D129" s="6"/>
       <c r="F129">
@@ -3914,7 +3920,7 @@
         <v>2</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D130" s="6"/>
       <c r="F130">
@@ -3936,7 +3942,7 @@
         <v>2</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D131" s="6"/>
       <c r="F131">
@@ -3958,7 +3964,7 @@
         <v>2</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D132" s="6"/>
       <c r="F132">
@@ -3980,7 +3986,7 @@
         <v>2</v>
       </c>
       <c r="C133" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D133" s="6"/>
       <c r="F133">
@@ -4002,7 +4008,7 @@
         <v>1</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D134" s="6"/>
       <c r="F134">
@@ -4024,7 +4030,7 @@
         <v>5</v>
       </c>
       <c r="C135" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D135" s="6"/>
       <c r="F135">
@@ -4046,7 +4052,7 @@
         <v>1</v>
       </c>
       <c r="C136" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D136" s="6"/>
       <c r="F136">
@@ -4068,7 +4074,7 @@
         <v>0</v>
       </c>
       <c r="C137" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D137" s="6"/>
       <c r="F137">
@@ -4090,18 +4096,18 @@
         <v>1</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D138" s="6"/>
       <c r="F138">
         <v>387</v>
       </c>
       <c r="G138">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I138" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.3">
@@ -4112,7 +4118,7 @@
         <v>2</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D139" s="6"/>
       <c r="F139">
@@ -4134,7 +4140,7 @@
         <v>3</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D140" s="6"/>
       <c r="F140">
@@ -4156,7 +4162,7 @@
         <v>1</v>
       </c>
       <c r="C141" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D141" s="6"/>
       <c r="F141">
@@ -4178,7 +4184,7 @@
         <v>1</v>
       </c>
       <c r="C142" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D142" s="6"/>
       <c r="F142">
@@ -4200,7 +4206,7 @@
         <v>1</v>
       </c>
       <c r="C143" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D143" s="6"/>
       <c r="F143">
@@ -4222,7 +4228,7 @@
         <v>4</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D144" s="6"/>
       <c r="F144">
@@ -4244,7 +4250,7 @@
         <v>5</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D145" s="6"/>
       <c r="F145">
@@ -4451,11 +4457,11 @@
         <v>435</v>
       </c>
       <c r="G155">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I155" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.3">
@@ -4531,11 +4537,11 @@
         <v>443</v>
       </c>
       <c r="G159">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I159" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.3">
@@ -4891,11 +4897,11 @@
         <v>495</v>
       </c>
       <c r="G177">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I177" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.3">
@@ -4931,11 +4937,11 @@
         <v>506</v>
       </c>
       <c r="G179">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I179" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.3">
@@ -4991,11 +4997,11 @@
         <v>509</v>
       </c>
       <c r="G182">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I182" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.3">
@@ -5231,11 +5237,11 @@
         <v>544</v>
       </c>
       <c r="G194">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I194" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.3">
@@ -5331,11 +5337,11 @@
         <v>555</v>
       </c>
       <c r="G199">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I199" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.3">
@@ -5611,11 +5617,11 @@
         <v>598</v>
       </c>
       <c r="G213">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I213" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.3">
@@ -5831,11 +5837,11 @@
         <v>621</v>
       </c>
       <c r="G224">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I224" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.3">
@@ -5971,11 +5977,11 @@
         <v>650</v>
       </c>
       <c r="G231">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I231" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.3">
@@ -6291,11 +6297,11 @@
         <v>700</v>
       </c>
       <c r="G247">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I247" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.3">
@@ -6311,11 +6317,11 @@
         <v>705</v>
       </c>
       <c r="G248">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I248" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.3">
@@ -7431,11 +7437,11 @@
         <v>874</v>
       </c>
       <c r="G304">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I304" s="6" t="str">
         <f t="shared" si="4"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="305" spans="1:9" x14ac:dyDescent="0.3">
@@ -7971,11 +7977,11 @@
         <v>978</v>
       </c>
       <c r="G331">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I331" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="332" spans="1:9" x14ac:dyDescent="0.3">
@@ -8251,11 +8257,11 @@
         <v>1027</v>
       </c>
       <c r="G345">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I345" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="346" spans="1:9" x14ac:dyDescent="0.3">
@@ -8351,11 +8357,11 @@
         <v>1037</v>
       </c>
       <c r="G350">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I350" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="351" spans="1:9" x14ac:dyDescent="0.3">
@@ -9371,11 +9377,11 @@
         <v>1195</v>
       </c>
       <c r="G401">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I401" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="402" spans="1:9" x14ac:dyDescent="0.3">
@@ -9391,11 +9397,11 @@
         <v>1196</v>
       </c>
       <c r="G402">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I402" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="403" spans="1:9" x14ac:dyDescent="0.3">
@@ -9411,11 +9417,11 @@
         <v>1200</v>
       </c>
       <c r="G403">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I403" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="404" spans="1:9" x14ac:dyDescent="0.3">
@@ -10571,11 +10577,11 @@
         <v>1381</v>
       </c>
       <c r="G461">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I461" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="462" spans="1:9" x14ac:dyDescent="0.3">
@@ -10591,11 +10597,11 @@
         <v>1391</v>
       </c>
       <c r="G462">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I462" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="463" spans="1:9" x14ac:dyDescent="0.3">
@@ -10831,11 +10837,11 @@
         <v>1426</v>
       </c>
       <c r="G474">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I474" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="475" spans="1:9" x14ac:dyDescent="0.3">
@@ -11091,11 +11097,11 @@
         <v>1472</v>
       </c>
       <c r="G487">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I487" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="488" spans="1:9" x14ac:dyDescent="0.3">
@@ -11331,11 +11337,11 @@
         <v>1507</v>
       </c>
       <c r="G499">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I499" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="500" spans="1:9" x14ac:dyDescent="0.3">
@@ -11711,11 +11717,11 @@
         <v>1566</v>
       </c>
       <c r="G518">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I518" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="519" spans="1:9" x14ac:dyDescent="0.3">
@@ -12131,11 +12137,11 @@
         <v>1653</v>
       </c>
       <c r="G539">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I539" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="540" spans="1:9" x14ac:dyDescent="0.3">
@@ -12251,11 +12257,11 @@
         <v>1672</v>
       </c>
       <c r="G545">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I545" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="546" spans="1:9" x14ac:dyDescent="0.3">
@@ -12471,11 +12477,11 @@
         <v>1710</v>
       </c>
       <c r="G556">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I556" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.3">
@@ -13111,11 +13117,11 @@
         <v>1809</v>
       </c>
       <c r="G588">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I588" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="589" spans="1:9" x14ac:dyDescent="0.3">
@@ -13231,11 +13237,11 @@
         <v>1829</v>
       </c>
       <c r="G594">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I594" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="595" spans="1:9" x14ac:dyDescent="0.3">
@@ -13611,11 +13617,11 @@
         <v>1883</v>
       </c>
       <c r="G613">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I613" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="614" spans="1:9" x14ac:dyDescent="0.3">
@@ -13731,11 +13737,11 @@
         <v>1911</v>
       </c>
       <c r="G619">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I619" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="620" spans="1:9" x14ac:dyDescent="0.3">
@@ -13751,11 +13757,11 @@
         <v>1912</v>
       </c>
       <c r="G620">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I620" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="621" spans="1:9" x14ac:dyDescent="0.3">
@@ -14531,11 +14537,11 @@
         <v>2028</v>
       </c>
       <c r="G659">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I659" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="660" spans="1:9" x14ac:dyDescent="0.3">
@@ -15091,11 +15097,11 @@
         <v>2153</v>
       </c>
       <c r="G687">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I687" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="688" spans="1:9" x14ac:dyDescent="0.3">
@@ -15211,11 +15217,11 @@
         <v>2164</v>
       </c>
       <c r="G693">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I693" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="694" spans="1:9" x14ac:dyDescent="0.3">
@@ -15511,11 +15517,11 @@
         <v>2216</v>
       </c>
       <c r="G708">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I708" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="709" spans="1:9" x14ac:dyDescent="0.3">
@@ -16011,11 +16017,11 @@
         <v>2293</v>
       </c>
       <c r="G733">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I733" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="734" spans="1:9" x14ac:dyDescent="0.3">
@@ -16411,11 +16417,11 @@
         <v>2354</v>
       </c>
       <c r="G753">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I753" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="754" spans="1:9" x14ac:dyDescent="0.3">
@@ -17051,11 +17057,11 @@
         <v>2448</v>
       </c>
       <c r="G785">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I785" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="786" spans="1:9" x14ac:dyDescent="0.3">
@@ -17251,11 +17257,11 @@
         <v>2484</v>
       </c>
       <c r="G795">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I795" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="796" spans="1:9" x14ac:dyDescent="0.3">
@@ -17391,11 +17397,11 @@
         <v>2498</v>
       </c>
       <c r="G802">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I802" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="803" spans="1:9" x14ac:dyDescent="0.3">
@@ -18731,11 +18737,11 @@
         <v>2702</v>
       </c>
       <c r="G869">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I869" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="870" spans="1:9" x14ac:dyDescent="0.3">
@@ -18831,11 +18837,11 @@
         <v>2714</v>
       </c>
       <c r="G874">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I874" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="875" spans="1:9" x14ac:dyDescent="0.3">
@@ -19251,11 +19257,11 @@
         <v>2783</v>
       </c>
       <c r="G895">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I895" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="896" spans="1:9" x14ac:dyDescent="0.3">
@@ -19411,11 +19417,11 @@
         <v>2802</v>
       </c>
       <c r="G903">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I903" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="904" spans="1:9" x14ac:dyDescent="0.3">
@@ -19711,11 +19717,11 @@
         <v>2830</v>
       </c>
       <c r="G918">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I918" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="919" spans="1:9" x14ac:dyDescent="0.3">
@@ -19871,11 +19877,11 @@
         <v>2852</v>
       </c>
       <c r="G926">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I926" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="927" spans="1:9" x14ac:dyDescent="0.3">
@@ -20231,11 +20237,11 @@
         <v>2907</v>
       </c>
       <c r="G944">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I944" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="945" spans="1:9" x14ac:dyDescent="0.3">
@@ -20811,11 +20817,11 @@
         <v>2975</v>
       </c>
       <c r="G973">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I973" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="974" spans="1:9" x14ac:dyDescent="0.3">
@@ -20891,11 +20897,11 @@
         <v>2994</v>
       </c>
       <c r="G977">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I977" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="978" spans="1:9" x14ac:dyDescent="0.3">
@@ -20931,11 +20937,11 @@
         <v>3008</v>
       </c>
       <c r="G979">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I979" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="980" spans="1:9" x14ac:dyDescent="0.3">
@@ -21111,11 +21117,11 @@
         <v>3044</v>
       </c>
       <c r="G988">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I988" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="989" spans="1:9" x14ac:dyDescent="0.3">
@@ -21191,11 +21197,11 @@
         <v>3057</v>
       </c>
       <c r="G992">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I992" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="993" spans="1:9" x14ac:dyDescent="0.3">
@@ -21251,11 +21257,11 @@
         <v>3075</v>
       </c>
       <c r="G995">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I995" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="996" spans="1:9" x14ac:dyDescent="0.3">
@@ -21291,11 +21297,11 @@
         <v>3079</v>
       </c>
       <c r="G997">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I997" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="998" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Improved readiblity of the  model's log
</commit_message>
<xml_diff>
--- a/compareOP.xlsx
+++ b/compareOP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DUT\Ki 2\Edge AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E64CC8D-0935-4854-B2C3-17FA4CC13C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40BD07DF-5F38-49F9-B4FA-FDBB0027BC0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56603411-7B59-498E-88B9-7E9448248F05}"/>
   </bookViews>
@@ -163,10 +163,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1480,11 +1480,11 @@
         <f t="shared" si="0"/>
         <v>F</v>
       </c>
-      <c r="O19" s="10" t="s">
+      <c r="O19" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="9"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="6">

</xml_diff>

<commit_message>
End of the day
</commit_message>
<xml_diff>
--- a/compareOP.xlsx
+++ b/compareOP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DUT\Ki 2\Edge AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{029F255C-2BC4-4443-9276-66A8FD30EB0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EDB4B5-321A-4460-8171-A431E2C19E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{56603411-7B59-498E-88B9-7E9448248F05}"/>
   </bookViews>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="L2" s="4">
         <f>COUNTIF(I2:I1001, "T")</f>
-        <v>957</v>
+        <v>836</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="L3" s="4">
         <f>L2/1000*100</f>
-        <v>95.7</v>
+        <v>83.6</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
@@ -1135,7 +1135,7 @@
         <v>14</v>
       </c>
       <c r="G5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -1363,11 +1363,11 @@
         <v>51</v>
       </c>
       <c r="G15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I15" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1463,11 +1463,11 @@
         <v>59</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I19" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
       <c r="O19" s="10" t="s">
         <v>7</v>
@@ -1489,7 +1489,7 @@
         <v>63</v>
       </c>
       <c r="G20">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -1510,11 +1510,11 @@
         <v>67</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I21" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
@@ -1552,11 +1552,11 @@
         <v>70</v>
       </c>
       <c r="G23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I23" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
@@ -1636,11 +1636,11 @@
         <v>87</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I27" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
@@ -1678,11 +1678,11 @@
         <v>93</v>
       </c>
       <c r="G29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I29" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
@@ -1867,7 +1867,7 @@
         <v>123</v>
       </c>
       <c r="G38">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -1993,11 +1993,11 @@
         <v>144</v>
       </c>
       <c r="G44">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I44" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -2161,11 +2161,11 @@
         <v>170</v>
       </c>
       <c r="G52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I52" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
@@ -2224,11 +2224,11 @@
         <v>175</v>
       </c>
       <c r="G55">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I55" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
@@ -2329,11 +2329,11 @@
         <v>183</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I60" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
@@ -2476,11 +2476,11 @@
         <v>199</v>
       </c>
       <c r="G67">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I67" s="6" t="str">
         <f t="shared" ref="I67:I130" si="1">IF(B67=G67, "T", "F")</f>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
@@ -2539,7 +2539,7 @@
         <v>210</v>
       </c>
       <c r="G70">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I70" s="6" t="str">
         <f t="shared" si="1"/>
@@ -2938,11 +2938,11 @@
         <v>251</v>
       </c>
       <c r="G89">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I89" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.3">
@@ -3127,11 +3127,11 @@
         <v>270</v>
       </c>
       <c r="G98">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I98" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.3">
@@ -3169,11 +3169,11 @@
         <v>276</v>
       </c>
       <c r="G100">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I100" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.3">
@@ -3379,11 +3379,11 @@
         <v>299</v>
       </c>
       <c r="G110">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I110" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.3">
@@ -3547,11 +3547,11 @@
         <v>324</v>
       </c>
       <c r="G118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I118" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.3">
@@ -3631,7 +3631,7 @@
         <v>340</v>
       </c>
       <c r="G122">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I122" s="6" t="str">
         <f t="shared" si="1"/>
@@ -3967,11 +3967,11 @@
         <v>387</v>
       </c>
       <c r="G138">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I138" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.3">
@@ -4135,11 +4135,11 @@
         <v>415</v>
       </c>
       <c r="G146">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I146" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.3">
@@ -4219,11 +4219,11 @@
         <v>423</v>
       </c>
       <c r="G150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I150" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.3">
@@ -4240,11 +4240,11 @@
         <v>424</v>
       </c>
       <c r="G151">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I151" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.3">
@@ -4324,7 +4324,7 @@
         <v>435</v>
       </c>
       <c r="G155">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I155" s="6" t="str">
         <f t="shared" si="2"/>
@@ -4345,11 +4345,11 @@
         <v>436</v>
       </c>
       <c r="G156">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I156" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.3">
@@ -4408,11 +4408,11 @@
         <v>443</v>
       </c>
       <c r="G159">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I159" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.3">
@@ -4429,11 +4429,11 @@
         <v>445</v>
       </c>
       <c r="G160">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I160" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.3">
@@ -4555,11 +4555,11 @@
         <v>461</v>
       </c>
       <c r="G166">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I166" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.3">
@@ -4786,11 +4786,11 @@
         <v>495</v>
       </c>
       <c r="G177">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I177" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.3">
@@ -4828,11 +4828,11 @@
         <v>506</v>
       </c>
       <c r="G179">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I179" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.3">
@@ -4849,11 +4849,11 @@
         <v>507</v>
       </c>
       <c r="G180">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I180" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.3">
@@ -4891,11 +4891,11 @@
         <v>509</v>
       </c>
       <c r="G182">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I182" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.3">
@@ -5059,11 +5059,11 @@
         <v>535</v>
       </c>
       <c r="G190">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I190" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.3">
@@ -5227,11 +5227,11 @@
         <v>554</v>
       </c>
       <c r="G198">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I198" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.3">
@@ -5332,11 +5332,11 @@
         <v>565</v>
       </c>
       <c r="G203">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I203" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.3">
@@ -5353,11 +5353,11 @@
         <v>567</v>
       </c>
       <c r="G204">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I204" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.3">
@@ -5542,7 +5542,7 @@
         <v>598</v>
       </c>
       <c r="G213">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I213" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5752,11 +5752,11 @@
         <v>620</v>
       </c>
       <c r="G223">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I223" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.3">
@@ -5773,7 +5773,7 @@
         <v>621</v>
       </c>
       <c r="G224">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I224" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5794,11 +5794,11 @@
         <v>626</v>
       </c>
       <c r="G225">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I225" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.3">
@@ -5899,11 +5899,11 @@
         <v>647</v>
       </c>
       <c r="G230">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I230" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.3">
@@ -5920,7 +5920,7 @@
         <v>650</v>
       </c>
       <c r="G231">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I231" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5962,11 +5962,11 @@
         <v>655</v>
       </c>
       <c r="G233">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I233" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.3">
@@ -6025,11 +6025,11 @@
         <v>670</v>
       </c>
       <c r="G236">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I236" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.3">
@@ -6088,11 +6088,11 @@
         <v>678</v>
       </c>
       <c r="G239">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I239" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.3">
@@ -6193,11 +6193,11 @@
         <v>691</v>
       </c>
       <c r="G244">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I244" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.3">
@@ -6256,11 +6256,11 @@
         <v>700</v>
       </c>
       <c r="G247">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I247" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.3">
@@ -6277,11 +6277,11 @@
         <v>705</v>
       </c>
       <c r="G248">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I248" s="6" t="str">
         <f t="shared" si="3"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.3">
@@ -6508,11 +6508,11 @@
         <v>755</v>
       </c>
       <c r="G259">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I259" s="6" t="str">
         <f t="shared" ref="I259:I322" si="4">IF(B259=G259, "T", "F")</f>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="260" spans="1:9" x14ac:dyDescent="0.3">
@@ -7327,7 +7327,7 @@
         <v>859</v>
       </c>
       <c r="G298">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I298" s="6" t="str">
         <f t="shared" si="4"/>
@@ -7915,11 +7915,11 @@
         <v>952</v>
       </c>
       <c r="G326">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I326" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="327" spans="1:9" x14ac:dyDescent="0.3">
@@ -7936,11 +7936,11 @@
         <v>962</v>
       </c>
       <c r="G327">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I327" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="328" spans="1:9" x14ac:dyDescent="0.3">
@@ -8020,7 +8020,7 @@
         <v>978</v>
       </c>
       <c r="G331">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I331" s="6" t="str">
         <f t="shared" si="5"/>
@@ -8314,11 +8314,11 @@
         <v>1027</v>
       </c>
       <c r="G345">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I345" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="346" spans="1:9" x14ac:dyDescent="0.3">
@@ -8419,11 +8419,11 @@
         <v>1037</v>
       </c>
       <c r="G350">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I350" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="351" spans="1:9" x14ac:dyDescent="0.3">
@@ -8608,11 +8608,11 @@
         <v>1061</v>
       </c>
       <c r="G359">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I359" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="360" spans="1:9" x14ac:dyDescent="0.3">
@@ -8734,11 +8734,11 @@
         <v>1078</v>
       </c>
       <c r="G365">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I365" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="366" spans="1:9" x14ac:dyDescent="0.3">
@@ -8839,11 +8839,11 @@
         <v>1091</v>
       </c>
       <c r="G370">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I370" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="371" spans="1:9" x14ac:dyDescent="0.3">
@@ -9028,11 +9028,11 @@
         <v>1113</v>
       </c>
       <c r="G379">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I379" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="380" spans="1:9" x14ac:dyDescent="0.3">
@@ -9154,11 +9154,11 @@
         <v>1128</v>
       </c>
       <c r="G385">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I385" s="6" t="str">
         <f t="shared" si="5"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="386" spans="1:9" x14ac:dyDescent="0.3">
@@ -9217,11 +9217,11 @@
         <v>1135</v>
       </c>
       <c r="G388">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I388" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="389" spans="1:9" x14ac:dyDescent="0.3">
@@ -9238,11 +9238,11 @@
         <v>1149</v>
       </c>
       <c r="G389">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I389" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="390" spans="1:9" x14ac:dyDescent="0.3">
@@ -9469,11 +9469,11 @@
         <v>1188</v>
       </c>
       <c r="G400">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I400" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="401" spans="1:9" x14ac:dyDescent="0.3">
@@ -9490,11 +9490,11 @@
         <v>1195</v>
       </c>
       <c r="G401">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I401" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="402" spans="1:9" x14ac:dyDescent="0.3">
@@ -9511,11 +9511,11 @@
         <v>1196</v>
       </c>
       <c r="G402">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I402" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="403" spans="1:9" x14ac:dyDescent="0.3">
@@ -9532,7 +9532,7 @@
         <v>1200</v>
       </c>
       <c r="G403">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I403" s="6" t="str">
         <f t="shared" si="6"/>
@@ -9658,11 +9658,11 @@
         <v>1213</v>
       </c>
       <c r="G409">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I409" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="410" spans="1:9" x14ac:dyDescent="0.3">
@@ -9679,11 +9679,11 @@
         <v>1216</v>
       </c>
       <c r="G410">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I410" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="411" spans="1:9" x14ac:dyDescent="0.3">
@@ -10120,11 +10120,11 @@
         <v>1270</v>
       </c>
       <c r="G431">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I431" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="432" spans="1:9" x14ac:dyDescent="0.3">
@@ -10204,11 +10204,11 @@
         <v>1286</v>
       </c>
       <c r="G435">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I435" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="436" spans="1:9" x14ac:dyDescent="0.3">
@@ -10372,11 +10372,11 @@
         <v>1309</v>
       </c>
       <c r="G443">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I443" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="444" spans="1:9" x14ac:dyDescent="0.3">
@@ -10435,11 +10435,11 @@
         <v>1320</v>
       </c>
       <c r="G446">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I446" s="6" t="str">
         <f t="shared" si="6"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="447" spans="1:9" x14ac:dyDescent="0.3">
@@ -10855,11 +10855,11 @@
         <v>1398</v>
       </c>
       <c r="G466">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I466" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="467" spans="1:9" x14ac:dyDescent="0.3">
@@ -10897,7 +10897,7 @@
         <v>1407</v>
       </c>
       <c r="G468">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I468" s="6" t="str">
         <f t="shared" si="7"/>
@@ -10939,11 +10939,11 @@
         <v>1413</v>
       </c>
       <c r="G470">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I470" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="471" spans="1:9" x14ac:dyDescent="0.3">
@@ -11002,11 +11002,11 @@
         <v>1422</v>
       </c>
       <c r="G473">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I473" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="474" spans="1:9" x14ac:dyDescent="0.3">
@@ -11023,11 +11023,11 @@
         <v>1426</v>
       </c>
       <c r="G474">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I474" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="475" spans="1:9" x14ac:dyDescent="0.3">
@@ -11296,11 +11296,11 @@
         <v>1472</v>
       </c>
       <c r="G487">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I487" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="488" spans="1:9" x14ac:dyDescent="0.3">
@@ -11317,11 +11317,11 @@
         <v>1474</v>
       </c>
       <c r="G488">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I488" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="489" spans="1:9" x14ac:dyDescent="0.3">
@@ -11401,11 +11401,11 @@
         <v>1483</v>
       </c>
       <c r="G492">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I492" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="493" spans="1:9" x14ac:dyDescent="0.3">
@@ -11590,11 +11590,11 @@
         <v>1510</v>
       </c>
       <c r="G501">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I501" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="502" spans="1:9" x14ac:dyDescent="0.3">
@@ -11632,11 +11632,11 @@
         <v>1512</v>
       </c>
       <c r="G503">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I503" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="504" spans="1:9" x14ac:dyDescent="0.3">
@@ -11779,11 +11779,11 @@
         <v>1538</v>
       </c>
       <c r="G510">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I510" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="511" spans="1:9" x14ac:dyDescent="0.3">
@@ -11863,11 +11863,11 @@
         <v>1554</v>
       </c>
       <c r="G514">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I514" s="6" t="str">
         <f t="shared" si="7"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="515" spans="1:9" x14ac:dyDescent="0.3">
@@ -12409,11 +12409,11 @@
         <v>1655</v>
       </c>
       <c r="G540">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I540" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="541" spans="1:9" x14ac:dyDescent="0.3">
@@ -12451,11 +12451,11 @@
         <v>1659</v>
       </c>
       <c r="G542">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I542" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="543" spans="1:9" x14ac:dyDescent="0.3">
@@ -12745,11 +12745,11 @@
         <v>1710</v>
       </c>
       <c r="G556">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I556" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.3">
@@ -12829,11 +12829,11 @@
         <v>1718</v>
       </c>
       <c r="G560">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I560" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="561" spans="1:9" x14ac:dyDescent="0.3">
@@ -12892,11 +12892,11 @@
         <v>1725</v>
       </c>
       <c r="G563">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I563" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="564" spans="1:9" x14ac:dyDescent="0.3">
@@ -12934,11 +12934,11 @@
         <v>1730</v>
       </c>
       <c r="G565">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I565" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="566" spans="1:9" x14ac:dyDescent="0.3">
@@ -12955,11 +12955,11 @@
         <v>1731</v>
       </c>
       <c r="G566">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I566" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="567" spans="1:9" x14ac:dyDescent="0.3">
@@ -12976,11 +12976,11 @@
         <v>1735</v>
       </c>
       <c r="G567">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I567" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="568" spans="1:9" x14ac:dyDescent="0.3">
@@ -12997,11 +12997,11 @@
         <v>1736</v>
       </c>
       <c r="G568">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I568" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="569" spans="1:9" x14ac:dyDescent="0.3">
@@ -13039,11 +13039,11 @@
         <v>1741</v>
       </c>
       <c r="G570">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I570" s="6" t="str">
         <f t="shared" si="8"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="571" spans="1:9" x14ac:dyDescent="0.3">
@@ -13417,7 +13417,7 @@
         <v>1809</v>
       </c>
       <c r="G588">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I588" s="6" t="str">
         <f t="shared" si="9"/>
@@ -13543,11 +13543,11 @@
         <v>1829</v>
       </c>
       <c r="G594">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I594" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="595" spans="1:9" x14ac:dyDescent="0.3">
@@ -13942,11 +13942,11 @@
         <v>1883</v>
       </c>
       <c r="G613">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I613" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="614" spans="1:9" x14ac:dyDescent="0.3">
@@ -14005,11 +14005,11 @@
         <v>1896</v>
       </c>
       <c r="G616">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I616" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="617" spans="1:9" x14ac:dyDescent="0.3">
@@ -14068,7 +14068,7 @@
         <v>1911</v>
       </c>
       <c r="G619">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I619" s="6" t="str">
         <f t="shared" si="9"/>
@@ -14089,7 +14089,7 @@
         <v>1912</v>
       </c>
       <c r="G620">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I620" s="6" t="str">
         <f t="shared" si="9"/>
@@ -14152,11 +14152,11 @@
         <v>1924</v>
       </c>
       <c r="G623">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I623" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="624" spans="1:9" x14ac:dyDescent="0.3">
@@ -14215,11 +14215,11 @@
         <v>1933</v>
       </c>
       <c r="G626">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I626" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="627" spans="1:9" x14ac:dyDescent="0.3">
@@ -14320,11 +14320,11 @@
         <v>1941</v>
       </c>
       <c r="G631">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I631" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="632" spans="1:9" x14ac:dyDescent="0.3">
@@ -14341,11 +14341,11 @@
         <v>1950</v>
       </c>
       <c r="G632">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I632" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="633" spans="1:9" x14ac:dyDescent="0.3">
@@ -14509,11 +14509,11 @@
         <v>1966</v>
       </c>
       <c r="G640">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I640" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="641" spans="1:9" x14ac:dyDescent="0.3">
@@ -14614,11 +14614,11 @@
         <v>1980</v>
       </c>
       <c r="G645">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I645" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="646" spans="1:9" x14ac:dyDescent="0.3">
@@ -14740,11 +14740,11 @@
         <v>2005</v>
       </c>
       <c r="G651">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I651" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="652" spans="1:9" x14ac:dyDescent="0.3">
@@ -14824,11 +14824,11 @@
         <v>2014</v>
       </c>
       <c r="G655">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I655" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="656" spans="1:9" x14ac:dyDescent="0.3">
@@ -14845,11 +14845,11 @@
         <v>2015</v>
       </c>
       <c r="G656">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I656" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="657" spans="1:9" x14ac:dyDescent="0.3">
@@ -14887,7 +14887,7 @@
         <v>2025</v>
       </c>
       <c r="G658">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I658" s="6" t="str">
         <f t="shared" si="10"/>
@@ -15181,11 +15181,11 @@
         <v>2073</v>
       </c>
       <c r="G672">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I672" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="673" spans="1:9" x14ac:dyDescent="0.3">
@@ -15349,11 +15349,11 @@
         <v>2119</v>
       </c>
       <c r="G680">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I680" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="681" spans="1:9" x14ac:dyDescent="0.3">
@@ -15454,11 +15454,11 @@
         <v>2138</v>
       </c>
       <c r="G685">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I685" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="686" spans="1:9" x14ac:dyDescent="0.3">
@@ -15496,11 +15496,11 @@
         <v>2153</v>
       </c>
       <c r="G687">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I687" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="688" spans="1:9" x14ac:dyDescent="0.3">
@@ -15580,11 +15580,11 @@
         <v>2162</v>
       </c>
       <c r="G691">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I691" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="692" spans="1:9" x14ac:dyDescent="0.3">
@@ -15601,11 +15601,11 @@
         <v>2163</v>
       </c>
       <c r="G692">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I692" s="6" t="str">
         <f t="shared" si="10"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="693" spans="1:9" x14ac:dyDescent="0.3">
@@ -15622,7 +15622,7 @@
         <v>2164</v>
       </c>
       <c r="G693">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I693" s="6" t="str">
         <f t="shared" si="10"/>
@@ -15916,7 +15916,7 @@
         <v>2212</v>
       </c>
       <c r="G707">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I707" s="6" t="str">
         <f t="shared" ref="I707:I770" si="11">IF(B707=G707, "T", "F")</f>
@@ -16021,11 +16021,11 @@
         <v>2227</v>
       </c>
       <c r="G712">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I712" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="713" spans="1:9" x14ac:dyDescent="0.3">
@@ -16084,11 +16084,11 @@
         <v>2234</v>
       </c>
       <c r="G715">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I715" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="716" spans="1:9" x14ac:dyDescent="0.3">
@@ -16294,11 +16294,11 @@
         <v>2259</v>
       </c>
       <c r="G725">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I725" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="726" spans="1:9" x14ac:dyDescent="0.3">
@@ -16483,11 +16483,11 @@
         <v>2295</v>
       </c>
       <c r="G734">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I734" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="735" spans="1:9" x14ac:dyDescent="0.3">
@@ -16504,11 +16504,11 @@
         <v>2298</v>
       </c>
       <c r="G735">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I735" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="736" spans="1:9" x14ac:dyDescent="0.3">
@@ -16525,11 +16525,11 @@
         <v>2299</v>
       </c>
       <c r="G736">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I736" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="737" spans="1:9" x14ac:dyDescent="0.3">
@@ -16567,11 +16567,11 @@
         <v>2303</v>
       </c>
       <c r="G738">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I738" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="739" spans="1:9" x14ac:dyDescent="0.3">
@@ -16756,11 +16756,11 @@
         <v>2340</v>
       </c>
       <c r="G747">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I747" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="748" spans="1:9" x14ac:dyDescent="0.3">
@@ -16798,11 +16798,11 @@
         <v>2346</v>
       </c>
       <c r="G749">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I749" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="750" spans="1:9" x14ac:dyDescent="0.3">
@@ -16819,11 +16819,11 @@
         <v>2347</v>
       </c>
       <c r="G750">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I750" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="751" spans="1:9" x14ac:dyDescent="0.3">
@@ -16987,11 +16987,11 @@
         <v>2362</v>
       </c>
       <c r="G758">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I758" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="759" spans="1:9" x14ac:dyDescent="0.3">
@@ -17050,11 +17050,11 @@
         <v>2369</v>
       </c>
       <c r="G761">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I761" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="762" spans="1:9" x14ac:dyDescent="0.3">
@@ -17197,11 +17197,11 @@
         <v>2390</v>
       </c>
       <c r="G768">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I768" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="769" spans="1:9" x14ac:dyDescent="0.3">
@@ -17218,11 +17218,11 @@
         <v>2397</v>
       </c>
       <c r="G769">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I769" s="6" t="str">
         <f t="shared" si="11"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="770" spans="1:9" x14ac:dyDescent="0.3">
@@ -17428,11 +17428,11 @@
         <v>2425</v>
       </c>
       <c r="G779">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I779" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="780" spans="1:9" x14ac:dyDescent="0.3">
@@ -17470,11 +17470,11 @@
         <v>2431</v>
       </c>
       <c r="G781">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I781" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="782" spans="1:9" x14ac:dyDescent="0.3">
@@ -17512,11 +17512,11 @@
         <v>2439</v>
       </c>
       <c r="G783">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I783" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="784" spans="1:9" x14ac:dyDescent="0.3">
@@ -17554,11 +17554,11 @@
         <v>2448</v>
       </c>
       <c r="G785">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I785" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="786" spans="1:9" x14ac:dyDescent="0.3">
@@ -17743,11 +17743,11 @@
         <v>2482</v>
       </c>
       <c r="G794">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I794" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="795" spans="1:9" x14ac:dyDescent="0.3">
@@ -17764,11 +17764,11 @@
         <v>2484</v>
       </c>
       <c r="G795">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I795" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="796" spans="1:9" x14ac:dyDescent="0.3">
@@ -18184,11 +18184,11 @@
         <v>2530</v>
       </c>
       <c r="G815">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I815" s="6" t="str">
         <f t="shared" si="12"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="816" spans="1:9" x14ac:dyDescent="0.3">
@@ -18688,7 +18688,7 @@
         <v>2609</v>
       </c>
       <c r="G839">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I839" s="6" t="str">
         <f t="shared" si="13"/>
@@ -18856,11 +18856,11 @@
         <v>2639</v>
       </c>
       <c r="G847">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I847" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="848" spans="1:9" x14ac:dyDescent="0.3">
@@ -18919,11 +18919,11 @@
         <v>2648</v>
       </c>
       <c r="G850">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I850" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="851" spans="1:9" x14ac:dyDescent="0.3">
@@ -18940,11 +18940,11 @@
         <v>2650</v>
       </c>
       <c r="G851">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I851" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>F</v>
+        <v>T</v>
       </c>
     </row>
     <row r="852" spans="1:9" x14ac:dyDescent="0.3">
@@ -19003,11 +19003,11 @@
         <v>2661</v>
       </c>
       <c r="G854">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I854" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="855" spans="1:9" x14ac:dyDescent="0.3">
@@ -19318,7 +19318,7 @@
         <v>2702</v>
       </c>
       <c r="G869">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I869" s="6" t="str">
         <f t="shared" si="13"/>
@@ -19465,11 +19465,11 @@
         <v>2718</v>
       </c>
       <c r="G876">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I876" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="877" spans="1:9" x14ac:dyDescent="0.3">
@@ -19486,11 +19486,11 @@
         <v>2721</v>
       </c>
       <c r="G877">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I877" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="878" spans="1:9" x14ac:dyDescent="0.3">
@@ -19654,11 +19654,11 @@
         <v>2748</v>
       </c>
       <c r="G885">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I885" s="6" t="str">
         <f t="shared" si="13"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="886" spans="1:9" x14ac:dyDescent="0.3">
@@ -20158,7 +20158,7 @@
         <v>2810</v>
       </c>
       <c r="G909">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I909" s="6" t="str">
         <f t="shared" si="14"/>
@@ -20347,11 +20347,11 @@
         <v>2830</v>
       </c>
       <c r="G918">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I918" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="919" spans="1:9" x14ac:dyDescent="0.3">
@@ -20515,7 +20515,7 @@
         <v>2852</v>
       </c>
       <c r="G926">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I926" s="6" t="str">
         <f t="shared" si="14"/>
@@ -20683,11 +20683,11 @@
         <v>2876</v>
       </c>
       <c r="G934">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I934" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="935" spans="1:9" x14ac:dyDescent="0.3">
@@ -20809,11 +20809,11 @@
         <v>2899</v>
       </c>
       <c r="G940">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I940" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="941" spans="1:9" x14ac:dyDescent="0.3">
@@ -20830,11 +20830,11 @@
         <v>2901</v>
       </c>
       <c r="G941">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I941" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="942" spans="1:9" x14ac:dyDescent="0.3">
@@ -20935,11 +20935,11 @@
         <v>2909</v>
       </c>
       <c r="G946">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I946" s="6" t="str">
         <f t="shared" si="14"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="947" spans="1:9" x14ac:dyDescent="0.3">
@@ -21460,11 +21460,11 @@
         <v>2969</v>
       </c>
       <c r="G971">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I971" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="972" spans="1:9" x14ac:dyDescent="0.3">
@@ -21502,11 +21502,11 @@
         <v>2975</v>
       </c>
       <c r="G973">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I973" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="974" spans="1:9" x14ac:dyDescent="0.3">
@@ -21523,11 +21523,11 @@
         <v>2976</v>
       </c>
       <c r="G974">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I974" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="975" spans="1:9" x14ac:dyDescent="0.3">
@@ -21586,11 +21586,11 @@
         <v>2994</v>
       </c>
       <c r="G977">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I977" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="978" spans="1:9" x14ac:dyDescent="0.3">
@@ -21607,11 +21607,11 @@
         <v>2995</v>
       </c>
       <c r="G978">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I978" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="979" spans="1:9" x14ac:dyDescent="0.3">
@@ -21691,11 +21691,11 @@
         <v>3015</v>
       </c>
       <c r="G982">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I982" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="983" spans="1:9" x14ac:dyDescent="0.3">
@@ -21712,11 +21712,11 @@
         <v>3016</v>
       </c>
       <c r="G983">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I983" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="984" spans="1:9" x14ac:dyDescent="0.3">
@@ -21817,11 +21817,11 @@
         <v>3044</v>
       </c>
       <c r="G988">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I988" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="989" spans="1:9" x14ac:dyDescent="0.3">
@@ -21901,11 +21901,11 @@
         <v>3057</v>
       </c>
       <c r="G992">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I992" s="6" t="str">
         <f t="shared" si="15"/>
-        <v>T</v>
+        <v>F</v>
       </c>
     </row>
     <row r="993" spans="1:9" x14ac:dyDescent="0.3">
@@ -22006,7 +22006,7 @@
         <v>3079</v>
       </c>
       <c r="G997">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I997" s="6" t="str">
         <f t="shared" si="15"/>

</xml_diff>